<commit_message>
Updated file on week 1 completed
</commit_message>
<xml_diff>
--- a/Intern_Training_Progress_Tracker.xlsx
+++ b/Intern_Training_Progress_Tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramya\OneDrive\Desktop\Internship Update\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramya\internship-training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41537C64-80BC-49C9-A7DE-6B98DB69BBFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A241E761-1098-42C8-93FB-256CFE2D5F7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="219">
   <si>
     <t>🚀  6-Week Intern Training Progress Tracker</t>
   </si>
@@ -699,6 +699,23 @@
 •	Logical operators: and, or, not
 •	Nesting conditions; common beginner mistakes (= vs ==, indentation)
 •	Reading input with input() and type conversion</t>
+  </si>
+  <si>
+    <t>•	Why loops exist: avoiding repetition
+•	for loops and the range() function
+•	while loops and loop conditions
+•	Loop control: break and continue
+•	Combining loops with conditionals; the accumulator pattern (sums, counts)</t>
+  </si>
+  <si>
+    <t>10.06.2026</t>
+  </si>
+  <si>
+    <t>•	Lists: creation, indexing, slicing, append/remove, iteration
+•	Dictionaries: key-value pairs, access, update, iteration
+•	Tuples and sets (brief); when to use each structure
+•	Functions: def, parameters, return values, scope
+•	Combining functions, loops, and data structures together</t>
   </si>
 </sst>
 </file>
@@ -895,7 +912,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -972,6 +989,12 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -996,10 +1019,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1318,32 +1338,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
     </row>
     <row r="2" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A4" s="1" t="s">
@@ -1378,18 +1398,18 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.7">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="29"/>
     </row>
     <row r="6" spans="1:10" ht="156.6" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A6" s="2">
@@ -1419,7 +1439,7 @@
       <c r="I6" s="2">
         <v>5</v>
       </c>
-      <c r="J6" s="36" t="s">
+      <c r="J6" s="27" t="s">
         <v>212</v>
       </c>
     </row>
@@ -1483,11 +1503,11 @@
       <c r="I8" s="2">
         <v>5</v>
       </c>
-      <c r="J8" s="35" t="s">
+      <c r="J8" s="26" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.65">
+    <row r="9" spans="1:10" ht="79.2" x14ac:dyDescent="0.65">
       <c r="A9" s="2">
         <v>4</v>
       </c>
@@ -1504,16 +1524,22 @@
         <v>25</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" s="2"/>
+        <v>210</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>214</v>
+      </c>
       <c r="H9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I9" s="2"/>
-      <c r="J9" s="3"/>
-    </row>
-    <row r="10" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.65">
+        <v>208</v>
+      </c>
+      <c r="I9" s="2">
+        <v>5</v>
+      </c>
+      <c r="J9" s="26" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="132" x14ac:dyDescent="0.65">
       <c r="A10" s="2">
         <v>5</v>
       </c>
@@ -1529,29 +1555,35 @@
       <c r="E10" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G10" s="2"/>
+      <c r="F10" s="37" t="s">
+        <v>210</v>
+      </c>
+      <c r="G10" s="37" t="s">
+        <v>217</v>
+      </c>
       <c r="H10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" s="2"/>
-      <c r="J10" s="3"/>
+        <v>208</v>
+      </c>
+      <c r="I10" s="2">
+        <v>4</v>
+      </c>
+      <c r="J10" s="26" t="s">
+        <v>218</v>
+      </c>
     </row>
     <row r="12" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="27"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="29"/>
+      <c r="I12" s="29"/>
+      <c r="J12" s="29"/>
     </row>
     <row r="13" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A13" s="4">
@@ -1684,18 +1716,18 @@
       <c r="J17" s="5"/>
     </row>
     <row r="19" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A19" s="29" t="s">
+      <c r="A19" s="31" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="27"/>
-      <c r="I19" s="27"/>
-      <c r="J19" s="27"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="29"/>
+      <c r="J19" s="29"/>
     </row>
     <row r="20" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A20" s="6">
@@ -1828,18 +1860,18 @@
       <c r="J24" s="7"/>
     </row>
     <row r="26" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A26" s="29" t="s">
+      <c r="A26" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="27"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="27"/>
-      <c r="F26" s="27"/>
-      <c r="G26" s="27"/>
-      <c r="H26" s="27"/>
-      <c r="I26" s="27"/>
-      <c r="J26" s="27"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="29"/>
+      <c r="H26" s="29"/>
+      <c r="I26" s="29"/>
+      <c r="J26" s="29"/>
     </row>
     <row r="27" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A27" s="8">
@@ -1972,18 +2004,18 @@
       <c r="J31" s="9"/>
     </row>
     <row r="33" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A33" s="29" t="s">
+      <c r="A33" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="B33" s="27"/>
-      <c r="C33" s="27"/>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
-      <c r="F33" s="27"/>
-      <c r="G33" s="27"/>
-      <c r="H33" s="27"/>
-      <c r="I33" s="27"/>
-      <c r="J33" s="27"/>
+      <c r="B33" s="29"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
+      <c r="H33" s="29"/>
+      <c r="I33" s="29"/>
+      <c r="J33" s="29"/>
     </row>
     <row r="34" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A34" s="10">
@@ -2116,18 +2148,18 @@
       <c r="J38" s="11"/>
     </row>
     <row r="40" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A40" s="29" t="s">
+      <c r="A40" s="31" t="s">
         <v>97</v>
       </c>
-      <c r="B40" s="27"/>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="27"/>
-      <c r="F40" s="27"/>
-      <c r="G40" s="27"/>
-      <c r="H40" s="27"/>
-      <c r="I40" s="27"/>
-      <c r="J40" s="27"/>
+      <c r="B40" s="29"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="29"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="29"/>
+      <c r="H40" s="29"/>
+      <c r="I40" s="29"/>
+      <c r="J40" s="29"/>
     </row>
     <row r="41" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A41" s="12">
@@ -2260,18 +2292,18 @@
       <c r="J45" s="13"/>
     </row>
     <row r="47" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A47" s="26" t="s">
+      <c r="A47" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="B47" s="27"/>
-      <c r="C47" s="27"/>
-      <c r="D47" s="27"/>
-      <c r="E47" s="27"/>
-      <c r="F47" s="27"/>
-      <c r="G47" s="27"/>
-      <c r="H47" s="27"/>
-      <c r="I47" s="27"/>
-      <c r="J47" s="27"/>
+      <c r="B47" s="29"/>
+      <c r="C47" s="29"/>
+      <c r="D47" s="29"/>
+      <c r="E47" s="29"/>
+      <c r="F47" s="29"/>
+      <c r="G47" s="29"/>
+      <c r="H47" s="29"/>
+      <c r="I47" s="29"/>
+      <c r="J47" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -2315,26 +2347,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="36" t="s">
         <v>115</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.65">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="34" t="s">
         <v>116</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
     </row>
     <row r="4" spans="1:7" ht="28.05" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A4" s="1" t="s">
@@ -2370,14 +2402,14 @@
         <v>5</v>
       </c>
       <c r="D5" s="2">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E5" s="14">
         <f t="shared" ref="E5:E11" si="0">IF(C5=0,0,D5/C5)</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>124</v>
+        <v>1</v>
+      </c>
+      <c r="F5" s="14">
+        <v>1</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>125</v>
@@ -2504,35 +2536,35 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A11" s="33" t="s">
+      <c r="A11" s="35" t="s">
         <v>136</v>
       </c>
-      <c r="B11" s="33"/>
+      <c r="B11" s="35"/>
       <c r="C11" s="20">
         <f>SUM(C5:C10)</f>
         <v>30</v>
       </c>
       <c r="D11" s="20">
         <f>SUM(D5:D10)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E11" s="21">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="F11" s="20"/>
       <c r="G11" s="20"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.65">
-      <c r="A13" s="31" t="s">
+      <c r="A13" s="33" t="s">
         <v>137</v>
       </c>
-      <c r="B13" s="27"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="27"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2558,22 +2590,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.95" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="36" t="s">
         <v>138</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
     </row>
     <row r="3" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="31" t="s">
         <v>139</v>
       </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
     </row>
     <row r="4" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A4" s="22" t="s">
@@ -2599,7 +2631,7 @@
       <c r="B5" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="37" t="s">
         <v>146</v>
       </c>
       <c r="D5" s="2"/>
@@ -2645,13 +2677,13 @@
       <c r="E8" s="2"/>
     </row>
     <row r="10" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A10" s="29" t="s">
+      <c r="A10" s="31" t="s">
         <v>150</v>
       </c>
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
     </row>
     <row r="11" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A11" s="22" t="s">
@@ -2723,13 +2755,13 @@
       <c r="E15" s="4"/>
     </row>
     <row r="17" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A17" s="29" t="s">
+      <c r="A17" s="31" t="s">
         <v>155</v>
       </c>
-      <c r="B17" s="27"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
     </row>
     <row r="18" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A18" s="22" t="s">
@@ -2801,13 +2833,13 @@
       <c r="E22" s="6"/>
     </row>
     <row r="24" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="31" t="s">
         <v>160</v>
       </c>
-      <c r="B24" s="27"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
+      <c r="B24" s="29"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="29"/>
     </row>
     <row r="25" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A25" s="22" t="s">
@@ -2879,13 +2911,13 @@
       <c r="E29" s="8"/>
     </row>
     <row r="31" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A31" s="29" t="s">
+      <c r="A31" s="31" t="s">
         <v>165</v>
       </c>
-      <c r="B31" s="27"/>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="27"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
     </row>
     <row r="32" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A32" s="22" t="s">
@@ -2957,13 +2989,13 @@
       <c r="E36" s="10"/>
     </row>
     <row r="38" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A38" s="29" t="s">
+      <c r="A38" s="31" t="s">
         <v>170</v>
       </c>
-      <c r="B38" s="27"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="27"/>
+      <c r="B38" s="29"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="29"/>
+      <c r="E38" s="29"/>
     </row>
     <row r="39" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.65">
       <c r="A39" s="22" t="s">
@@ -3062,7 +3094,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="31.95" customHeight="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="36" t="s">
         <v>175</v>
       </c>
     </row>
@@ -3195,12 +3227,12 @@
         <v>177</v>
       </c>
     </row>
-    <row r="29" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.65">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.65">
       <c r="A29" s="23" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="30" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.65">
+    <row r="30" spans="1:1" ht="26.4" x14ac:dyDescent="0.65">
       <c r="A30" s="23" t="s">
         <v>199</v>
       </c>

</xml_diff>